<commit_message>
Finalizar Taller 3 con grafico en Excel y bitacora actualizada
</commit_message>
<xml_diff>
--- a/data/raw/cotizaciones.xlsx
+++ b/data/raw/cotizaciones.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3b6ffb6eb20c50b6/Escritorio/Equipo_04_COMII/data/raw/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="4" documentId="8_{587725E5-EC58-4276-980F-8D0CAB1C09BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{68FCF821-E6D5-4B5E-8630-1A9D1480D9B3}"/>
+  <xr:revisionPtr revIDLastSave="5" documentId="8_{587725E5-EC58-4276-980F-8D0CAB1C09BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4036BCAB-3E08-45A7-9D11-76C06DD99259}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{75A8E435-5125-44DF-928C-D2C0D10B14F6}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" tabRatio="283" xr2:uid="{75A8E435-5125-44DF-928C-D2C0D10B14F6}"/>
   </bookViews>
   <sheets>
     <sheet name="Datos " sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="22">
   <si>
     <t>Producto</t>
   </si>
@@ -55,6 +55,42 @@
   </si>
   <si>
     <t>Proveedor</t>
+  </si>
+  <si>
+    <t>Laptop i17</t>
+  </si>
+  <si>
+    <t>Computadoras S.A</t>
+  </si>
+  <si>
+    <t>TechElSalvador</t>
+  </si>
+  <si>
+    <t>Monitor 27"</t>
+  </si>
+  <si>
+    <t>Importadora SV</t>
+  </si>
+  <si>
+    <t>Teclado y Mouse Inalámbrico</t>
+  </si>
+  <si>
+    <t>GlobalTech</t>
+  </si>
+  <si>
+    <t>CompraMax</t>
+  </si>
+  <si>
+    <t>Servidor NAS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DataSytem </t>
+  </si>
+  <si>
+    <t>Inversiones Digitales</t>
+  </si>
+  <si>
+    <t>Monitor 24"</t>
   </si>
 </sst>
 </file>
@@ -101,13 +137,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -115,11 +152,63 @@
     <cellStyle name="Moneda" xfId="1" builtinId="4"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="3">
+  <dxfs count="7">
     <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -129,6 +218,34 @@
         <strike val="0"/>
         <condense val="0"/>
         <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
         <outline val="0"/>
         <shadow val="0"/>
         <u val="none"/>
@@ -154,14 +271,14 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{2F0AD21E-7B71-4407-B8DF-9B369B81A98B}" name="Tabla1" displayName="Tabla1" ref="A1:E5" totalsRowShown="0">
-  <autoFilter ref="A1:E5" xr:uid="{2F0AD21E-7B71-4407-B8DF-9B369B81A98B}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{2F0AD21E-7B71-4407-B8DF-9B369B81A98B}" name="Tabla1" displayName="Tabla1" ref="A1:E20" totalsRowShown="0" headerRowDxfId="1" dataDxfId="0">
+  <autoFilter ref="A1:E20" xr:uid="{2F0AD21E-7B71-4407-B8DF-9B369B81A98B}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{33419652-7D9B-47B4-927B-C49D7FA54E9A}" name="Producto"/>
-    <tableColumn id="2" xr3:uid="{EFA3B42E-DA0B-46FB-8DEB-478052390E64}" name="Proveedor"/>
-    <tableColumn id="3" xr3:uid="{B687FC65-3CCF-46D6-A912-03AF74B5DBB2}" name="Precio" dataDxfId="2" dataCellStyle="Moneda"/>
-    <tableColumn id="4" xr3:uid="{C448CA62-16DB-4883-A965-469B608E7AB3}" name="PlazoEntrega" dataDxfId="1"/>
-    <tableColumn id="5" xr3:uid="{4D794EC6-7298-4240-9FD6-7521B0D4539A}" name="CondicionesPago" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{33419652-7D9B-47B4-927B-C49D7FA54E9A}" name="Producto" dataDxfId="6"/>
+    <tableColumn id="2" xr3:uid="{EFA3B42E-DA0B-46FB-8DEB-478052390E64}" name="Proveedor" dataDxfId="5"/>
+    <tableColumn id="3" xr3:uid="{B687FC65-3CCF-46D6-A912-03AF74B5DBB2}" name="Precio" dataDxfId="4" dataCellStyle="Moneda"/>
+    <tableColumn id="4" xr3:uid="{C448CA62-16DB-4883-A965-469B608E7AB3}" name="PlazoEntrega" dataDxfId="3"/>
+    <tableColumn id="5" xr3:uid="{4D794EC6-7298-4240-9FD6-7521B0D4539A}" name="CondicionesPago" dataDxfId="2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight15" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -464,100 +581,369 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C39A4C9F-7D13-4E51-876E-3DAA88306E16}">
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="24.140625" customWidth="1"/>
-    <col min="2" max="2" width="17.28515625" customWidth="1"/>
+    <col min="1" max="1" width="27" customWidth="1"/>
+    <col min="2" max="2" width="20" customWidth="1"/>
     <col min="3" max="3" width="12.85546875" customWidth="1"/>
     <col min="4" max="4" width="14.5703125" customWidth="1"/>
     <col min="5" max="5" width="18.28515625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="2" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+      <c r="A2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="2" t="s">
         <v>5</v>
       </c>
       <c r="C2" s="1">
         <v>650</v>
       </c>
-      <c r="D2" s="2">
+      <c r="D2" s="3">
         <v>5</v>
       </c>
-      <c r="E2" s="3">
+      <c r="E2" s="4">
         <v>30</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+      <c r="A3" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="2" t="s">
         <v>6</v>
       </c>
       <c r="C3" s="1">
         <v>620</v>
       </c>
-      <c r="D3" s="3">
+      <c r="D3" s="4">
         <v>10</v>
       </c>
-      <c r="E3" s="3">
+      <c r="E3" s="4">
         <v>15</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+      <c r="A4" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="2" t="s">
         <v>5</v>
       </c>
       <c r="C4" s="1">
         <v>180</v>
       </c>
-      <c r="D4" s="3">
+      <c r="D4" s="4">
         <v>3</v>
       </c>
-      <c r="E4" s="3">
+      <c r="E4" s="4">
         <v>30</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
+      <c r="A5" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C5" s="1">
         <v>195</v>
       </c>
-      <c r="D5" s="3">
+      <c r="D5" s="4">
         <v>2</v>
       </c>
-      <c r="E5" s="3">
+      <c r="E5" s="4">
         <v>45</v>
       </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C6" s="1">
+        <v>850</v>
+      </c>
+      <c r="D6" s="4">
+        <v>5</v>
+      </c>
+      <c r="E6" s="4">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C7" s="1">
+        <v>820</v>
+      </c>
+      <c r="D7" s="4">
+        <v>10</v>
+      </c>
+      <c r="E7" s="4">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C8" s="1">
+        <v>175</v>
+      </c>
+      <c r="D8" s="4">
+        <v>7</v>
+      </c>
+      <c r="E8" s="4">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C9" s="1">
+        <v>130</v>
+      </c>
+      <c r="D9" s="4">
+        <v>1</v>
+      </c>
+      <c r="E9" s="4">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C10" s="1">
+        <v>45</v>
+      </c>
+      <c r="D10" s="4">
+        <v>4</v>
+      </c>
+      <c r="E10" s="4">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C11" s="1">
+        <v>30</v>
+      </c>
+      <c r="D11" s="4">
+        <v>3</v>
+      </c>
+      <c r="E11" s="4">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C12" s="1">
+        <v>28</v>
+      </c>
+      <c r="D12" s="4">
+        <v>15</v>
+      </c>
+      <c r="E12" s="4">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A13" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C13" s="1">
+        <v>32</v>
+      </c>
+      <c r="D13" s="4">
+        <v>20</v>
+      </c>
+      <c r="E13" s="4">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A14" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C14" s="1">
+        <v>1000</v>
+      </c>
+      <c r="D14" s="4">
+        <v>30</v>
+      </c>
+      <c r="E14" s="4">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A15" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C15" s="1">
+        <v>1400</v>
+      </c>
+      <c r="D15" s="4">
+        <v>10</v>
+      </c>
+      <c r="E15" s="4">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A16" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C16" s="1">
+        <v>1200</v>
+      </c>
+      <c r="D16" s="4">
+        <v>15</v>
+      </c>
+      <c r="E16" s="4">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A17" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C17" s="1">
+        <v>130</v>
+      </c>
+      <c r="D17" s="4">
+        <v>4</v>
+      </c>
+      <c r="E17" s="4">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A18" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C18" s="1">
+        <v>150</v>
+      </c>
+      <c r="D18" s="4">
+        <v>1</v>
+      </c>
+      <c r="E18" s="4">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A19" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C19" s="1">
+        <v>145</v>
+      </c>
+      <c r="D19" s="4">
+        <v>3</v>
+      </c>
+      <c r="E19" s="4">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A20" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C20" s="1">
+        <v>170</v>
+      </c>
+      <c r="D20" s="4">
+        <v>2</v>
+      </c>
+      <c r="E20" s="4">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A21" s="2"/>
+      <c r="B21" s="2"/>
+      <c r="C21" s="2"/>
+      <c r="D21" s="2"/>
+      <c r="E21" s="2"/>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A22" s="2"/>
+      <c r="B22" s="2"/>
+      <c r="C22" s="2"/>
+      <c r="D22" s="2"/>
+      <c r="E22" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>